<commit_message>
Rename Jim and Wife to Chung Jim Huang and Yu Xi Huang.
Keep guest ids jim and jim-wife so seating-state table assignments stay put. Add the couple to the RSVP export so a regenerate does not drop the names.

Co-authored-by: Skdvnn <Skdvnn@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/rsvp-export.xlsx
+++ b/data/rsvp-export.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1197" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="187">
   <si>
     <t/>
   </si>
@@ -567,6 +567,12 @@
   </si>
   <si>
     <t>Zheng</t>
+  </si>
+  <si>
+    <t>Chung Jim</t>
+  </si>
+  <si>
+    <t>Yu Xi</t>
   </si>
 </sst>
 </file>
@@ -611,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F115"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="4.40625" customWidth="true" bestFit="true"/>
@@ -2922,6 +2928,46 @@
         <v>64</v>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B116" t="s" s="0">
+        <v>185</v>
+      </c>
+      <c r="C116" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="D116" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="E116" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F116" t="s" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B117" t="s" s="0">
+        <v>186</v>
+      </c>
+      <c r="C117" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="D117" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F117" t="s" s="0">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Rename Jim and Wife to Chung Jim Huang and Yu Xi Huang. (#1)
Keep guest ids jim and jim-wife so seating-state table assignments stay put. Add the couple to the RSVP export so a regenerate does not drop the names.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: Skdvnn <Skdvnn@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/rsvp-export.xlsx
+++ b/data/rsvp-export.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1197" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="187">
   <si>
     <t/>
   </si>
@@ -567,6 +567,12 @@
   </si>
   <si>
     <t>Zheng</t>
+  </si>
+  <si>
+    <t>Chung Jim</t>
+  </si>
+  <si>
+    <t>Yu Xi</t>
   </si>
 </sst>
 </file>
@@ -611,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F115"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="4.40625" customWidth="true" bestFit="true"/>
@@ -2922,6 +2928,46 @@
         <v>64</v>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B116" t="s" s="0">
+        <v>185</v>
+      </c>
+      <c r="C116" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="D116" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="E116" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F116" t="s" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B117" t="s" s="0">
+        <v>186</v>
+      </c>
+      <c r="C117" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="D117" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F117" t="s" s="0">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>